<commit_message>
Updated a few things
</commit_message>
<xml_diff>
--- a/314e-ig/output/StructureDefinition-carePlan-activity-targetDateTime.xlsx
+++ b/314e-ig/output/StructureDefinition-carePlan-activity-targetDateTime.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-11T14:17:09+05:30</t>
+    <t>2026-06-18T13:36:33+05:30</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,8 +84,7 @@
     <t>Applied to an individual activity element within a CarePlan resource.
 Stores the target or goal date-time for completing that specific care plan
 activity.
-Standard FHIR CarePlan.activity has no dedicated target date field separate
-from scheduledTiming or scheduledPeriod.</t>
+Note that the targetDateTime is separate from CarePlan.activity.scheduled[x].</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>